<commit_message>
Add UP_05 Camber Bracket FEA workflow and baseline FST15 data
</commit_message>
<xml_diff>
--- a/FST16_Assemblies_Export_DL.xlsx
+++ b/FST16_Assemblies_Export_DL.xlsx
@@ -46,11 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -128,20 +125,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AssembliesTable" displayName="AssembliesTable" ref="A1:E5" headerRowCount="1">
-  <autoFilter ref="A1:E5"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Assembly Version"/>
-    <tableColumn id="2" name="Date"/>
-    <tableColumn id="3" name="Total Weight (g)"/>
-    <tableColumn id="4" name="Description"/>
-    <tableColumn id="5" name="Part Configuration"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -471,25 +454,25 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>2026-10-12 22:02:36</t>
         </is>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" t="n">
         <v>1690.22</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>The first iteration for the new motors where the bearings sit right on top of the seal</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>TD: v1.2
 HB_01: v1
@@ -503,25 +486,25 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>2.0 (Without Support)</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>2026-10-13 20:49:23</t>
         </is>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" t="n">
         <v>648.28</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>This assembly has the objective of having a comparative analysis with the FST15 design with the same features, focusing in the new v2.0 transmission</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>TD: v2.0
 UP_01: v2.0 (without supports)
@@ -533,25 +516,25 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>FST15 (Without Support)</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>2026-10-13 20:44:41</t>
         </is>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" t="n">
         <v>856.61</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>This assembly has the objective of having a comparative baseline without the supports</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>UP_01: vFST15 (without supports)
 UP_02: vFST15 (with all features)
@@ -563,30 +546,31 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>FST15</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>2026-10-18 10:53:30</t>
         </is>
       </c>
-      <c r="C5" s="1" t="n">
-        <v>2220.16</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="C5" t="n">
+        <v>2270.05</v>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>FST15 Baseline</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>HB_01: vFST15
 UP_01: vFST15
 UP_02: vFST15
 UP_03: vFST15
+UP_05: vFST15
 Inner Bearing: v61815
 Outer Bearing: v61815
 Seal: v85X100X9 HMSA10 V</t>
@@ -595,8 +579,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>